<commit_message>
lock account, attendance, enrollment
fix lỗi lock acc, done chức năng attendance, comment code enrollment đợi sửa db
</commit_message>
<xml_diff>
--- a/students_import2.xlsx
+++ b/students_import2.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26827"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\FPT\Sem9-SP26\SEP\EDUCEN-SEP490-\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DEFAULT\FPT\SEP-G58\Code\EDUCEN-SEP490-\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC619A51-2F18-4DAE-A1ED-D873049F4338}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="students_import" sheetId="1" r:id="rId1"/>
@@ -23,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="181">
   <si>
     <t>Username</t>
   </si>
@@ -557,12 +556,21 @@
   </si>
   <si>
     <t>test057@gmail.com</t>
+  </si>
+  <si>
+    <t>nguyen van 58</t>
+  </si>
+  <si>
+    <t>test058@gmai.com</t>
+  </si>
+  <si>
+    <t>test058</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1388,19 +1396,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.88671875" customWidth="1"/>
-    <col min="2" max="2" width="31.109375" customWidth="1"/>
-    <col min="3" max="3" width="33.88671875" customWidth="1"/>
-    <col min="4" max="4" width="37.44140625" customWidth="1"/>
-    <col min="5" max="5" width="17.88671875" customWidth="1"/>
-    <col min="6" max="6" width="32.6640625" customWidth="1"/>
+    <col min="1" max="1" width="20.85546875" customWidth="1"/>
+    <col min="2" max="2" width="31.140625" customWidth="1"/>
+    <col min="3" max="3" width="33.85546875" customWidth="1"/>
+    <col min="4" max="4" width="37.42578125" customWidth="1"/>
+    <col min="5" max="5" width="17.85546875" customWidth="1"/>
+    <col min="6" max="6" width="32.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1423,7 +1431,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1446,7 +1454,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -1469,7 +1477,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1492,7 +1500,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -1515,7 +1523,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -1544,19 +1552,19 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88768A2A-C4B2-4A5B-B985-03C8CBA6A2F0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="33.33203125" customWidth="1"/>
-    <col min="3" max="3" width="35.33203125" customWidth="1"/>
-    <col min="4" max="4" width="25.44140625" customWidth="1"/>
-    <col min="5" max="5" width="21.5546875" customWidth="1"/>
-    <col min="6" max="6" width="36.21875" customWidth="1"/>
-    <col min="7" max="7" width="22.5546875" customWidth="1"/>
+    <col min="2" max="2" width="33.28515625" customWidth="1"/>
+    <col min="3" max="3" width="35.28515625" customWidth="1"/>
+    <col min="4" max="4" width="25.42578125" customWidth="1"/>
+    <col min="5" max="5" width="21.5703125" customWidth="1"/>
+    <col min="6" max="6" width="36.28515625" customWidth="1"/>
+    <col min="7" max="7" width="22.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1579,7 +1587,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>29</v>
       </c>
@@ -1602,7 +1610,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -1625,7 +1633,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -1648,7 +1656,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>39</v>
       </c>
@@ -1671,7 +1679,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>42</v>
       </c>
@@ -1694,7 +1702,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>45</v>
       </c>
@@ -1717,7 +1725,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>48</v>
       </c>
@@ -1740,7 +1748,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>51</v>
       </c>
@@ -1763,7 +1771,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>54</v>
       </c>
@@ -1786,7 +1794,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>57</v>
       </c>
@@ -1815,11 +1823,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06953985-C075-4BB3-A447-6CAD8C73ED67}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1842,7 +1850,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>60</v>
       </c>
@@ -1865,7 +1873,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>63</v>
       </c>
@@ -1888,7 +1896,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>66</v>
       </c>
@@ -1911,7 +1919,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>70</v>
       </c>
@@ -1934,7 +1942,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>73</v>
       </c>
@@ -1957,7 +1965,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>76</v>
       </c>
@@ -1980,7 +1988,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>79</v>
       </c>
@@ -2003,7 +2011,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>82</v>
       </c>
@@ -2026,7 +2034,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>85</v>
       </c>
@@ -2049,7 +2057,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>88</v>
       </c>
@@ -2078,17 +2086,17 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64CBD805-FB40-4F13-A6A5-BD6B0B460E94}">
-  <dimension ref="A1:G28"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G29"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="37.88671875" customWidth="1"/>
-    <col min="3" max="3" width="28.6640625" customWidth="1"/>
-    <col min="4" max="4" width="35.44140625" customWidth="1"/>
-    <col min="6" max="6" width="38.77734375" customWidth="1"/>
+    <col min="2" max="2" width="37.85546875" customWidth="1"/>
+    <col min="3" max="3" width="28.7109375" customWidth="1"/>
+    <col min="4" max="4" width="35.42578125" customWidth="1"/>
+    <col min="6" max="6" width="38.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2111,7 +2119,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>91</v>
       </c>
@@ -2134,7 +2142,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>94</v>
       </c>
@@ -2157,7 +2165,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>98</v>
       </c>
@@ -2180,7 +2188,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>102</v>
       </c>
@@ -2203,7 +2211,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>105</v>
       </c>
@@ -2226,7 +2234,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>108</v>
       </c>
@@ -2249,7 +2257,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>111</v>
       </c>
@@ -2272,7 +2280,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>114</v>
       </c>
@@ -2295,7 +2303,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>117</v>
       </c>
@@ -2318,7 +2326,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>120</v>
       </c>
@@ -2341,7 +2349,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>123</v>
       </c>
@@ -2364,7 +2372,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>129</v>
       </c>
@@ -2387,7 +2395,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>132</v>
       </c>
@@ -2410,7 +2418,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>135</v>
       </c>
@@ -2433,7 +2441,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>138</v>
       </c>
@@ -2456,7 +2464,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>143</v>
       </c>
@@ -2479,7 +2487,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>127</v>
       </c>
@@ -2502,7 +2510,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>148</v>
       </c>
@@ -2525,7 +2533,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>151</v>
       </c>
@@ -2548,7 +2556,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>154</v>
       </c>
@@ -2571,7 +2579,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>157</v>
       </c>
@@ -2594,7 +2602,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>160</v>
       </c>
@@ -2617,7 +2625,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>163</v>
       </c>
@@ -2640,7 +2648,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>164</v>
       </c>
@@ -2663,7 +2671,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>169</v>
       </c>
@@ -2686,7 +2694,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>172</v>
       </c>
@@ -2709,7 +2717,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>173</v>
       </c>
@@ -2729,28 +2737,52 @@
         <v>47490</v>
       </c>
       <c r="G28" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>180</v>
+      </c>
+      <c r="B29" t="s">
+        <v>178</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="D29">
+        <v>123456789</v>
+      </c>
+      <c r="E29" t="s">
+        <v>27</v>
+      </c>
+      <c r="F29" s="1">
+        <v>44197</v>
+      </c>
+      <c r="G29" t="s">
         <v>15</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="20" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="C12" r:id="rId1" xr:uid="{9EF190BC-0467-4877-BDA3-177A138B607B}"/>
-    <hyperlink ref="C13" r:id="rId2" xr:uid="{89DE7E01-0A64-4289-8807-B84637E752FD}"/>
-    <hyperlink ref="C14" r:id="rId3" xr:uid="{C0D218DE-2F58-40E6-83A1-FB1B0DDA9DA5}"/>
-    <hyperlink ref="C15" r:id="rId4" xr:uid="{564B7280-3EDC-402C-91DA-1307B66F6985}"/>
-    <hyperlink ref="C16" r:id="rId5" xr:uid="{9F56D980-05B6-4792-ADC3-6EFA175EB89D}"/>
-    <hyperlink ref="C17" r:id="rId6" xr:uid="{E4D3471D-F9CE-4DA0-868F-37730E5AB38B}"/>
-    <hyperlink ref="C19" r:id="rId7" xr:uid="{90634BFB-4A53-4CEE-A673-BC336AF85C1F}"/>
-    <hyperlink ref="C20" r:id="rId8" xr:uid="{FB8A14CE-0B74-48EB-A26F-2CAA0D3B713B}"/>
-    <hyperlink ref="C21" r:id="rId9" xr:uid="{DEBABF58-F010-4D52-A9C9-403A7AB9F353}"/>
-    <hyperlink ref="C22" r:id="rId10" xr:uid="{8FE31751-3312-497E-B731-893F6E49876D}"/>
-    <hyperlink ref="C23" r:id="rId11" xr:uid="{B81D7015-BAC5-4C49-AA4C-80FC86294A29}"/>
-    <hyperlink ref="C24" r:id="rId12" xr:uid="{EC71B839-4E18-4EFA-B457-0531E5B6DF30}"/>
-    <hyperlink ref="C25" r:id="rId13" xr:uid="{BCAF30E8-A778-4F43-9BB6-228A99FC951D}"/>
-    <hyperlink ref="C26" r:id="rId14" xr:uid="{16E75220-659F-4EA0-A2A7-FF324E21E93F}"/>
-    <hyperlink ref="C27" r:id="rId15" xr:uid="{8D15BD03-5795-487D-9D3C-224F5F77ACD6}"/>
-    <hyperlink ref="C28" r:id="rId16" xr:uid="{825467AF-FFAF-4782-A436-AFC37B9ECFFE}"/>
+    <hyperlink ref="C12" r:id="rId1"/>
+    <hyperlink ref="C13" r:id="rId2"/>
+    <hyperlink ref="C14" r:id="rId3"/>
+    <hyperlink ref="C15" r:id="rId4"/>
+    <hyperlink ref="C16" r:id="rId5"/>
+    <hyperlink ref="C17" r:id="rId6"/>
+    <hyperlink ref="C19" r:id="rId7"/>
+    <hyperlink ref="C20" r:id="rId8"/>
+    <hyperlink ref="C21" r:id="rId9"/>
+    <hyperlink ref="C22" r:id="rId10"/>
+    <hyperlink ref="C23" r:id="rId11"/>
+    <hyperlink ref="C24" r:id="rId12"/>
+    <hyperlink ref="C25" r:id="rId13"/>
+    <hyperlink ref="C26" r:id="rId14"/>
+    <hyperlink ref="C27" r:id="rId15"/>
+    <hyperlink ref="C28" r:id="rId16"/>
+    <hyperlink ref="C29" r:id="rId17"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
block upload, create active user + block access to inactive tenant
</commit_message>
<xml_diff>
--- a/students_import2.xlsx
+++ b/students_import2.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DEFAULT\FPT\SEP-G58\Code\EDUCEN-SEP490-\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEP490\EDUCEN-SEP490-\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C1B67A7-0D8B-4EC1-889A-DD1BA5B83A65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="students_import" sheetId="1" r:id="rId1"/>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="42">
   <si>
     <t>Username</t>
   </si>
@@ -109,12 +110,51 @@
   </si>
   <si>
     <t>PhoneNumber</t>
+  </si>
+  <si>
+    <t>ParentName</t>
+  </si>
+  <si>
+    <t>ParentPhone</t>
+  </si>
+  <si>
+    <t>ParentEmail</t>
+  </si>
+  <si>
+    <t>Nguyen Van B1</t>
+  </si>
+  <si>
+    <t>Nguyen Van C1</t>
+  </si>
+  <si>
+    <t>Nguyen Van D1</t>
+  </si>
+  <si>
+    <t>Nguyen Van E1</t>
+  </si>
+  <si>
+    <t>test0101@email.com</t>
+  </si>
+  <si>
+    <t>test0102@email.com</t>
+  </si>
+  <si>
+    <t>test0103@email.com</t>
+  </si>
+  <si>
+    <t>test0104@email.com</t>
+  </si>
+  <si>
+    <t>test0105@email.com</t>
+  </si>
+  <si>
+    <t>Nguyen Van A1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -940,19 +980,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" customWidth="1"/>
-    <col min="2" max="2" width="31.140625" customWidth="1"/>
-    <col min="3" max="3" width="33.85546875" customWidth="1"/>
-    <col min="4" max="4" width="37.42578125" customWidth="1"/>
-    <col min="5" max="5" width="17.85546875" customWidth="1"/>
-    <col min="6" max="6" width="32.7109375" customWidth="1"/>
+    <col min="1" max="1" width="20.88671875" customWidth="1"/>
+    <col min="2" max="2" width="31.109375" customWidth="1"/>
+    <col min="3" max="3" width="33.88671875" customWidth="1"/>
+    <col min="4" max="4" width="37.44140625" customWidth="1"/>
+    <col min="5" max="5" width="17.88671875" customWidth="1"/>
+    <col min="6" max="6" width="32.6640625" customWidth="1"/>
+    <col min="8" max="8" width="16.21875" customWidth="1"/>
+    <col min="9" max="9" width="21.21875" customWidth="1"/>
+    <col min="10" max="10" width="12.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -974,8 +1017,17 @@
       <c r="G1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -997,8 +1049,17 @@
       <c r="G2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H2" t="s">
+        <v>41</v>
+      </c>
+      <c r="I2">
+        <v>901234567</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -1020,8 +1081,17 @@
       <c r="G3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H3" t="s">
+        <v>32</v>
+      </c>
+      <c r="I3">
+        <v>901234568</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1043,8 +1113,17 @@
       <c r="G4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H4" t="s">
+        <v>33</v>
+      </c>
+      <c r="I4">
+        <v>901234569</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -1066,8 +1145,17 @@
       <c r="G5" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5">
+        <v>901234570</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -1089,54 +1177,70 @@
       <c r="G6" t="s">
         <v>10</v>
       </c>
+      <c r="H6" t="s">
+        <v>35</v>
+      </c>
+      <c r="I6">
+        <v>901234571</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>40</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="J2" r:id="rId1" xr:uid="{2AC31191-FD24-448D-8094-A415C1C7FE95}"/>
+    <hyperlink ref="J3" r:id="rId2" xr:uid="{DD89A9E3-226F-4FE1-93F7-5EAF20A11EB6}"/>
+    <hyperlink ref="J4" r:id="rId3" xr:uid="{E3DCE1B6-55C2-4B9B-A22D-12F3E704A35F}"/>
+    <hyperlink ref="J5" r:id="rId4" xr:uid="{BC778F77-80DB-4AE1-A7C5-A6054CC69B78}"/>
+    <hyperlink ref="J6" r:id="rId5" xr:uid="{2A0A3230-BEFA-4262-9FC4-EA1C4AACE30B}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="F2:F11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.28515625" customWidth="1"/>
-    <col min="2" max="2" width="33.28515625" customWidth="1"/>
-    <col min="3" max="3" width="35.28515625" customWidth="1"/>
-    <col min="4" max="4" width="35.5703125" customWidth="1"/>
-    <col min="5" max="5" width="21.5703125" customWidth="1"/>
-    <col min="6" max="6" width="36.28515625" customWidth="1"/>
-    <col min="7" max="7" width="22.5703125" customWidth="1"/>
+    <col min="1" max="1" width="22.33203125" customWidth="1"/>
+    <col min="2" max="2" width="33.33203125" customWidth="1"/>
+    <col min="3" max="3" width="35.33203125" customWidth="1"/>
+    <col min="4" max="4" width="35.5546875" customWidth="1"/>
+    <col min="5" max="5" width="21.5546875" customWidth="1"/>
+    <col min="6" max="6" width="36.33203125" customWidth="1"/>
+    <col min="7" max="7" width="22.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F2" s="1"/>
     </row>
-    <row r="3" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F3" s="1"/>
     </row>
-    <row r="4" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F4" s="1"/>
     </row>
-    <row r="5" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F5" s="1"/>
     </row>
-    <row r="6" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F6" s="1"/>
     </row>
-    <row r="7" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F7" s="1"/>
     </row>
-    <row r="8" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F8" s="1"/>
     </row>
-    <row r="9" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F9" s="1"/>
     </row>
-    <row r="10" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F10" s="1"/>
     </row>
-    <row r="11" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F11" s="1"/>
     </row>
   </sheetData>
@@ -1145,38 +1249,38 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="F2:F11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="2" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F2" s="1"/>
     </row>
-    <row r="3" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F3" s="1"/>
     </row>
-    <row r="4" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F4" s="1"/>
     </row>
-    <row r="5" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F5" s="1"/>
     </row>
-    <row r="6" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F6" s="1"/>
     </row>
-    <row r="7" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F7" s="1"/>
     </row>
-    <row r="8" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F8" s="1"/>
     </row>
-    <row r="9" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F9" s="1"/>
     </row>
-    <row r="10" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F10" s="1"/>
     </row>
-    <row r="11" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F11" s="1"/>
     </row>
   </sheetData>
@@ -1185,18 +1289,18 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G29"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="37.85546875" customWidth="1"/>
-    <col min="3" max="3" width="28.7109375" customWidth="1"/>
-    <col min="4" max="4" width="35.42578125" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" customWidth="1"/>
-    <col min="6" max="6" width="38.7109375" customWidth="1"/>
+    <col min="2" max="2" width="37.88671875" customWidth="1"/>
+    <col min="3" max="3" width="28.6640625" customWidth="1"/>
+    <col min="4" max="4" width="35.44140625" customWidth="1"/>
+    <col min="5" max="5" width="12.88671875" customWidth="1"/>
+    <col min="6" max="6" width="38.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="2"/>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1205,101 +1309,101 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F2" s="1"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F3" s="1"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F4" s="1"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F5" s="1"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F6" s="1"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F7" s="1"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F8" s="1"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F9" s="1"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F10" s="1"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="F11" s="1"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C12" s="3"/>
       <c r="F12" s="1"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C13" s="3"/>
       <c r="F13" s="1"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C14" s="3"/>
       <c r="F14" s="1"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C15" s="3"/>
       <c r="F15" s="1"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C16" s="3"/>
       <c r="F16" s="1"/>
     </row>
-    <row r="17" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="3:6" x14ac:dyDescent="0.3">
       <c r="C17" s="3"/>
       <c r="F17" s="1"/>
     </row>
-    <row r="19" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="3:6" x14ac:dyDescent="0.3">
       <c r="C19" s="3"/>
       <c r="F19" s="1"/>
     </row>
-    <row r="20" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="3:6" x14ac:dyDescent="0.3">
       <c r="C20" s="3"/>
       <c r="F20" s="1"/>
     </row>
-    <row r="21" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="3:6" x14ac:dyDescent="0.3">
       <c r="C21" s="3"/>
       <c r="F21" s="1"/>
     </row>
-    <row r="22" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="3:6" x14ac:dyDescent="0.3">
       <c r="C22" s="3"/>
       <c r="F22" s="1"/>
     </row>
-    <row r="23" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="3:6" x14ac:dyDescent="0.3">
       <c r="C23" s="3"/>
       <c r="F23" s="1"/>
     </row>
-    <row r="24" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="3:6" x14ac:dyDescent="0.3">
       <c r="C24" s="3"/>
       <c r="F24" s="1"/>
     </row>
-    <row r="25" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="3:6" x14ac:dyDescent="0.3">
       <c r="C25" s="3"/>
       <c r="F25" s="1"/>
     </row>
-    <row r="26" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="3:6" x14ac:dyDescent="0.3">
       <c r="C26" s="3"/>
       <c r="F26" s="1"/>
     </row>
-    <row r="27" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="3:6" x14ac:dyDescent="0.3">
       <c r="C27" s="3"/>
       <c r="F27" s="1"/>
     </row>
-    <row r="28" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="3:6" x14ac:dyDescent="0.3">
       <c r="C28" s="3"/>
       <c r="F28" s="1"/>
     </row>
-    <row r="29" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="3:6" x14ac:dyDescent="0.3">
       <c r="C29" s="3"/>
       <c r="F29" s="1"/>
     </row>

</xml_diff>